<commit_message>
feat(education-compass): point Deliveries at Schools instead of carrying school fields
A school application now names its school by School ID and nothing else; the name is maintained on
Schools and can be surfaced on the application with a lookup column, which stays outside the API
contract.

Dropping School Subject Ref along with the rest would have lost the organisation behind the
school, and the docx is explicit that a role id does not stand in for a subject id. Schools
therefore gains Subject Type and Subject Ref, the same separation Partners already makes: School ID
is the school role, Subject Ref is the organisation holding it.

Applied to the base: Schools gained the two columns and its timestamps became text, Deliveries
gained School ID. The three superseded columns are still on Deliveries, unreferenced - align never
deletes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phoenix Compass/education compass/tools/feishu-v05/Phoenix_Feishu_Operating_Model_V0.5.1_Master.xlsx
+++ b/Phoenix Compass/education compass/tools/feishu-v05/Phoenix_Feishu_Operating_Model_V0.5.1_Master.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D66"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D25" s="2" t="n"/>
     </row>
@@ -822,7 +822,7 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D27" s="2" t="n"/>
     </row>
@@ -1521,56 +1521,56 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Settlements</t>
+          <t>Applications</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Money Type</t>
+          <t>School Subject Ref</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>改名</t>
+          <t>丢弃</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>docx 指定用 Settlement Type 区分四类资金</t>
+          <t>机构主体 ID 移到 Schools.Subject Ref</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Settlements</t>
+          <t>Applications</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Business Basis Key</t>
+          <t>School Role Ref</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>丢弃</t>
+          <t>改名</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>底稿 Source Ref Type + Source Ref ID 已表达业务依据</t>
+          <t>改为引用 Schools.School ID</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Settlements</t>
+          <t>Applications</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Beneficiary / Counterparty ID</t>
+          <t>School Name</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>与 Counterparty Subject Ref 重复</t>
+          <t>学校名称只在 Schools 维护，申请侧可用查找列显示</t>
         </is>
       </c>
     </row>
@@ -1592,17 +1592,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Period Start</t>
+          <t>Money Type</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>采纳</t>
+          <t>改名</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>结算周期，底稿没有</t>
+          <t>docx 指定用 Settlement Type 区分四类资金</t>
         </is>
       </c>
     </row>
@@ -1614,37 +1614,103 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Period End</t>
+          <t>Business Basis Key</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>采纳</t>
+          <t>丢弃</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>底稿 Source Ref Type + Source Ref ID 已表达业务依据</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Beneficiary / Counterparty ID</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>丢弃</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>与 Counterparty Subject Ref 重复</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Period Start</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>采纳</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>结算周期，底稿没有</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Settlements</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Period End</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>采纳</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
           <t>Integration_Links</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>Source of Truth</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>采纳</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>docx 点名要求的列，底稿没有</t>
         </is>
@@ -1954,21 +2020,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1979,55 +2047,65 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
+          <t>Subject Type</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Subject Ref</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>School Code</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>School Name</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>School Type</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Cooperation Status</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Account Manager</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Agreement Ref</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Commission Eligible</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>Created At</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>Updated At</t>
         </is>
@@ -2041,55 +2119,68 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
+          <t>ORGANIZATION</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>ORG-REF-0001</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
           <t>SCH-HK-0001</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>示例大学</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>UNIVERSITY</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Katrina</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr"/>
-      <c r="I2" s="5" t="b">
+      <c r="J2" s="5" t="inlineStr"/>
+      <c r="K2" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="L2" s="5" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr"/>
-      <c r="L2" s="5" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr"/>
+      <c r="N2" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="4">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ORGANIZATION,PERSON"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"HIGH_SCHOOL,UNIVERSITY,GRADUATE_SCHOOL,OTHER"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PROSPECTING,NEGOTIATING,SIGNED,ACTIVE,PAUSED,TERMINATED"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ACTIVE,INACTIVE,DRAFT,ARCHIVED"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3785,7 +3876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV2"/>
+  <dimension ref="A1:AT2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3810,32 +3901,30 @@
     <col width="25" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="24" customWidth="1" min="23" max="23"/>
+    <col width="15" customWidth="1" min="23" max="23"/>
     <col width="21" customWidth="1" min="24" max="24"/>
-    <col width="17" customWidth="1" min="25" max="25"/>
-    <col width="21" customWidth="1" min="26" max="26"/>
-    <col width="14" customWidth="1" min="27" max="27"/>
-    <col width="23" customWidth="1" min="28" max="28"/>
-    <col width="24" customWidth="1" min="29" max="29"/>
-    <col width="20" customWidth="1" min="30" max="30"/>
-    <col width="26" customWidth="1" min="31" max="31"/>
-    <col width="16" customWidth="1" min="32" max="32"/>
-    <col width="18" customWidth="1" min="33" max="33"/>
-    <col width="24" customWidth="1" min="34" max="34"/>
-    <col width="32" customWidth="1" min="35" max="35"/>
-    <col width="18" customWidth="1" min="36" max="36"/>
-    <col width="16" customWidth="1" min="37" max="37"/>
-    <col width="20" customWidth="1" min="38" max="38"/>
-    <col width="22" customWidth="1" min="39" max="39"/>
-    <col width="31" customWidth="1" min="40" max="40"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="23" customWidth="1" min="26" max="26"/>
+    <col width="24" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="28" max="28"/>
+    <col width="26" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="24" customWidth="1" min="32" max="32"/>
+    <col width="32" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="16" customWidth="1" min="35" max="35"/>
+    <col width="20" customWidth="1" min="36" max="36"/>
+    <col width="22" customWidth="1" min="37" max="37"/>
+    <col width="31" customWidth="1" min="38" max="38"/>
+    <col width="14" customWidth="1" min="39" max="39"/>
+    <col width="20" customWidth="1" min="40" max="40"/>
     <col width="14" customWidth="1" min="41" max="41"/>
-    <col width="20" customWidth="1" min="42" max="42"/>
-    <col width="14" customWidth="1" min="43" max="43"/>
-    <col width="16" customWidth="1" min="44" max="44"/>
-    <col width="23" customWidth="1" min="45" max="45"/>
-    <col width="21" customWidth="1" min="46" max="46"/>
-    <col width="17" customWidth="1" min="47" max="47"/>
-    <col width="16" customWidth="1" min="48" max="48"/>
+    <col width="16" customWidth="1" min="42" max="42"/>
+    <col width="23" customWidth="1" min="43" max="43"/>
+    <col width="21" customWidth="1" min="44" max="44"/>
+    <col width="17" customWidth="1" min="45" max="45"/>
+    <col width="16" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3951,130 +4040,120 @@
       </c>
       <c r="W1" s="4" t="inlineStr">
         <is>
-          <t>School Subject Ref</t>
+          <t>School ID</t>
         </is>
       </c>
       <c r="X1" s="4" t="inlineStr">
         <is>
-          <t>School Role Ref</t>
+          <t>Program / Major</t>
         </is>
       </c>
       <c r="Y1" s="4" t="inlineStr">
         <is>
-          <t>School Name</t>
+          <t>Intake</t>
         </is>
       </c>
       <c r="Z1" s="4" t="inlineStr">
         <is>
-          <t>Program / Major</t>
+          <t>Application Round</t>
         </is>
       </c>
       <c r="AA1" s="4" t="inlineStr">
         <is>
-          <t>Intake</t>
+          <t>Application Status</t>
         </is>
       </c>
       <c r="AB1" s="4" t="inlineStr">
         <is>
-          <t>Application Round</t>
+          <t>Internal Owner</t>
         </is>
       </c>
       <c r="AC1" s="4" t="inlineStr">
         <is>
-          <t>Application Status</t>
+          <t>Data Package Version</t>
         </is>
       </c>
       <c r="AD1" s="4" t="inlineStr">
         <is>
-          <t>Internal Owner</t>
+          <t>Consent ID</t>
         </is>
       </c>
       <c r="AE1" s="4" t="inlineStr">
         <is>
-          <t>Data Package Version</t>
+          <t>Submitted At</t>
         </is>
       </c>
       <c r="AF1" s="4" t="inlineStr">
         <is>
-          <t>Consent ID</t>
+          <t>Submission Channel</t>
         </is>
       </c>
       <c r="AG1" s="4" t="inlineStr">
         <is>
-          <t>Submitted At</t>
+          <t>School Portal Ref / Receipt</t>
         </is>
       </c>
       <c r="AH1" s="4" t="inlineStr">
         <is>
-          <t>Submission Channel</t>
+          <t>Offer Status</t>
         </is>
       </c>
       <c r="AI1" s="4" t="inlineStr">
         <is>
-          <t>School Portal Ref / Receipt</t>
+          <t>Offer Date</t>
         </is>
       </c>
       <c r="AJ1" s="4" t="inlineStr">
         <is>
-          <t>Offer Status</t>
+          <t>Deposit Status</t>
         </is>
       </c>
       <c r="AK1" s="4" t="inlineStr">
         <is>
-          <t>Offer Date</t>
+          <t>Enrolment Status</t>
         </is>
       </c>
       <c r="AL1" s="4" t="inlineStr">
         <is>
-          <t>Deposit Status</t>
+          <t>School Commission Trigger</t>
         </is>
       </c>
       <c r="AM1" s="4" t="inlineStr">
         <is>
-          <t>Enrolment Status</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="AN1" s="4" t="inlineStr">
         <is>
-          <t>School Commission Trigger</t>
+          <t>Total Quantity</t>
         </is>
       </c>
       <c r="AO1" s="4" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="AP1" s="4" t="inlineStr">
         <is>
-          <t>Total Quantity</t>
+          <t>Updated At</t>
         </is>
       </c>
       <c r="AQ1" s="4" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Offer Received At</t>
         </is>
       </c>
       <c r="AR1" s="4" t="inlineStr">
         <is>
-          <t>Updated At</t>
+          <t>Deposit Paid At</t>
         </is>
       </c>
       <c r="AS1" s="4" t="inlineStr">
         <is>
-          <t>Offer Received At</t>
+          <t>Enrolled At</t>
         </is>
       </c>
       <c r="AT1" s="4" t="inlineStr">
-        <is>
-          <t>Deposit Paid At</t>
-        </is>
-      </c>
-      <c r="AU1" s="4" t="inlineStr">
-        <is>
-          <t>Enrolled At</t>
-        </is>
-      </c>
-      <c r="AV1" s="4" t="inlineStr">
         <is>
           <t>Created At</t>
         </is>
@@ -4171,69 +4250,61 @@
       </c>
       <c r="W2" s="5" t="inlineStr">
         <is>
-          <t>ORG-REF-0001</t>
+          <t>PN-SCH-0001</t>
         </is>
       </c>
       <c r="X2" s="5" t="inlineStr">
         <is>
-          <t>SCHOOL-ROLE-REF-0001</t>
+          <t>示例专业</t>
         </is>
       </c>
       <c r="Y2" s="5" t="inlineStr">
         <is>
-          <t>示例大学</t>
+          <t>2027-FALL</t>
         </is>
       </c>
       <c r="Z2" s="5" t="inlineStr">
         <is>
-          <t>示例专业</t>
+          <t>ROUND-1</t>
         </is>
       </c>
       <c r="AA2" s="5" t="inlineStr">
         <is>
-          <t>2027-FALL</t>
+          <t>DRAFT</t>
         </is>
       </c>
       <c r="AB2" s="5" t="inlineStr">
         <is>
-          <t>ROUND-1</t>
+          <t>Katrina</t>
         </is>
       </c>
       <c r="AC2" s="5" t="inlineStr">
         <is>
-          <t>DRAFT</t>
-        </is>
-      </c>
-      <c r="AD2" s="5" t="inlineStr">
-        <is>
-          <t>Katrina</t>
-        </is>
-      </c>
-      <c r="AE2" s="5" t="inlineStr">
-        <is>
           <t>1.0</t>
         </is>
       </c>
+      <c r="AD2" s="5" t="inlineStr"/>
+      <c r="AE2" s="5" t="inlineStr"/>
       <c r="AF2" s="5" t="inlineStr"/>
       <c r="AG2" s="5" t="inlineStr"/>
-      <c r="AH2" s="5" t="inlineStr"/>
+      <c r="AH2" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="AI2" s="5" t="inlineStr"/>
       <c r="AJ2" s="5" t="inlineStr">
         <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="AK2" s="5" t="inlineStr"/>
-      <c r="AL2" s="5" t="inlineStr">
-        <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="AM2" s="5" t="inlineStr">
+      <c r="AK2" s="5" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
+      <c r="AL2" s="5" t="inlineStr"/>
+      <c r="AM2" s="5" t="inlineStr"/>
       <c r="AN2" s="5" t="inlineStr"/>
       <c r="AO2" s="5" t="inlineStr"/>
       <c r="AP2" s="5" t="inlineStr"/>
@@ -4241,8 +4312,6 @@
       <c r="AR2" s="5" t="inlineStr"/>
       <c r="AS2" s="5" t="inlineStr"/>
       <c r="AT2" s="5" t="inlineStr"/>
-      <c r="AU2" s="5" t="inlineStr"/>
-      <c r="AV2" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="12">
@@ -4267,19 +4336,19 @@
     <dataValidation sqref="R2:R500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PENDING,PASS,FAIL,NOT_REQUIRED"</formula1>
     </dataValidation>
-    <dataValidation sqref="AC2:AC500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AA2:AA500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"DRAFT,WAITING_CLIENT,DATA_COMPLETE,READY_TO_SUBMIT,SUBMITTED,SCHOOL_ACKNOWLEDGED,OFFERED,REJECTED,WITHDRAWN,ENROLLED,CLOSED"</formula1>
     </dataValidation>
+    <dataValidation sqref="AF2:AF500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PORTAL,API,EMAIL,MANUAL,OTHER"</formula1>
+    </dataValidation>
     <dataValidation sqref="AH2:AH500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"PORTAL,API,EMAIL,MANUAL,OTHER"</formula1>
+      <formula1>"NONE,CONDITIONAL,UNCONDITIONAL,REJECTED,WAITLISTED,WITHDRAWN"</formula1>
     </dataValidation>
     <dataValidation sqref="AJ2:AJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"NONE,CONDITIONAL,UNCONDITIONAL,REJECTED,WAITLISTED,WITHDRAWN"</formula1>
-    </dataValidation>
-    <dataValidation sqref="AL2:AL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PENDING,PAID,WAIVED,NOT_REQUIRED,REFUNDED"</formula1>
     </dataValidation>
-    <dataValidation sqref="AM2:AM500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AK2:AK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PENDING,CONFIRMED,ENROLLED,DEFERRED,CANCELLED"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>